<commit_message>
Track account setup progress
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R75d658b381c34d09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Rae85baa8e61c4c7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Ra55ffd33155041d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R2c9fedb6d8df4418"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R221bc5da90ea4f00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7099a580ae0a4e63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Rc9009cf6318f482b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rfa2e59c568c64402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="Red6e6e1478e546b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R773b7fa9dc0e4352"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rda9787e55b3e40e6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6f421b0a8eaf4c4e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a43d444169343de"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9196686d4f2e4058"/>
 </x:worksheet>
 </file>
 
@@ -3608,7 +3608,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24e7a911ba334442"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e90605180ca4ac4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4285,7 +4285,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra402cc00379a45f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc140cce9bc984eae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4344,30 +4344,30 @@
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="9" t="str">
-        <x:v>Create Pinterest business account</x:v>
+        <x:v>Confirm Pinterest business account and rename profile</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
         <x:v>You</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Use US-English profile copy</x:v>
+        <x:v>Current profile: pinterest.com/davidforexe/</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="9" t="str">
-        <x:v>Create public GitHub repository</x:v>
+        <x:v>Make GitHub repository public</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>You + Codex</x:v>
+        <x:v>You</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Publish this starter site with GitHub Pages</x:v>
+        <x:v>Repository pushed; switch visibility to Public for GitHub Pages Free</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -4378,10 +4378,10 @@
         <x:v>You + Codex</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>Keep the github.io URL until $30 earned</x:v>
+        <x:v>Enable Pages from main / (root) after repository is public</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -4392,10 +4392,10 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
-        <x:v>Needs public profile URL</x:v>
+        <x:v>Temporary davidforexe URL added; update after rename</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -4490,7 +4490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9deff05682e84471"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R657bdb76a3c84cbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4775,7 +4775,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97f51fc15ba243d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33b69d99ac7f43ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Use live Pinterest brand profile
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7099a580ae0a4e63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Rc9009cf6318f482b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rfa2e59c568c64402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="Red6e6e1478e546b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R773b7fa9dc0e4352"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8488027bedf0494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="R800ce79de20e426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rae94f70a359640c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R7cc51b983c224dea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R2e2ac95565cb4882"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6f421b0a8eaf4c4e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1fcb4ea458e34799"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9196686d4f2e4058"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ffd5caae7b94fa1"/>
 </x:worksheet>
 </file>
 
@@ -3608,7 +3608,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e90605180ca4ac4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32bb2385f1d2430e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4285,7 +4285,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc140cce9bc984eae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cad13249d8b4b7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4350,10 +4350,10 @@
         <x:v>You</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Current profile: pinterest.com/davidforexe/</x:v>
+        <x:v>Live profile: pinterest.com/tidysmallspaces/</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -4395,7 +4395,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
-        <x:v>Temporary davidforexe URL added; update after rename</x:v>
+        <x:v>Live tidysmallspaces URL added</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -4490,7 +4490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R657bdb76a3c84cbc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd292fa9b4ee547d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4775,7 +4775,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33b69d99ac7f43ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a86d8b4da1547ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record live GitHub Pages launch
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8488027bedf0494e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="R800ce79de20e426c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rae94f70a359640c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R7cc51b983c224dea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R2e2ac95565cb4882"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R98444f79b2594c0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Rdf0ad9d4a3284c61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rd2edb1f4a4de4114"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R7e15489e149c4050"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="Ra992ddd50dcd480c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1fcb4ea458e34799"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R27d8c658ea8d4728"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ffd5caae7b94fa1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re45b367acb974722"/>
 </x:worksheet>
 </file>
 
@@ -3608,7 +3608,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32bb2385f1d2430e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc51f557c49b24047"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4285,7 +4285,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cad13249d8b4b7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c0252ce87444bce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4364,10 +4364,10 @@
         <x:v>You</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Repository pushed; switch visibility to Public for GitHub Pages Free</x:v>
+        <x:v>Public brand repository: davideskoundosincome/tidy-small-spaces</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -4378,10 +4378,10 @@
         <x:v>You + Codex</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>Enable Pages from main / (root) after repository is public</x:v>
+        <x:v>Live: davideskoundosincome.github.io/tidy-small-spaces/</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -4490,7 +4490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd292fa9b4ee547d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8ad0e957271446e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4775,7 +4775,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a86d8b4da1547ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2201d0a0bbe4fe4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Use clean Tidy Small Spaces website URL
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R98444f79b2594c0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Rdf0ad9d4a3284c61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rd2edb1f4a4de4114"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R7e15489e149c4050"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="Ra992ddd50dcd480c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5677c956106943fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Rf9cbd131a6ba444f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rd565ffb74e544775"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="Rf18a69cebdb24313"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R7ac5ed95f6934421"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R27d8c658ea8d4728"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R95ceb1f5f1ee4939"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re45b367acb974722"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58b019f6dce54bf2"/>
 </x:worksheet>
 </file>
 
@@ -3608,7 +3608,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc51f557c49b24047"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R120b70951f7e4965"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4285,7 +4285,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c0252ce87444bce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8757bf44b7014f0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4367,7 +4367,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Public brand repository: davideskoundosincome/tidy-small-spaces</x:v>
+        <x:v>Public brand repository: tidysmallspaces/tidysmallspaces.github.io</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -4381,7 +4381,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>Live: davideskoundosincome.github.io/tidy-small-spaces/</x:v>
+        <x:v>Live: tidysmallspaces.github.io/</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -4490,7 +4490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8ad0e957271446e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R231f82648b8c4dde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4775,7 +4775,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2201d0a0bbe4fe4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf96c643d4adb48dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add first upload-ready Pinterest batch
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5677c956106943fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Rf9cbd131a6ba444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rd565ffb74e544775"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="Rf18a69cebdb24313"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R7ac5ed95f6934421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R317fda558bce403f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Ra84ee8a9aded4499"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rdad84725b95248c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R4f8664acaae941df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="Rdfcdb76975034703"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R95ceb1f5f1ee4939"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd13a5605df244d07"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58b019f6dce54bf2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31cb536d6e3646d1"/>
 </x:worksheet>
 </file>
 
@@ -3608,7 +3608,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R120b70951f7e4965"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca9ec2e7bca14c52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4285,7 +4285,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8757bf44b7014f0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R373d89abc9354cd3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4445,13 +4445,13 @@
         <x:v>Create first weekly Pin batch</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>Together</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>14 original Pins</x:v>
+        <x:v>10 upload-ready PNGs plus editable SVG sources</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
@@ -4462,10 +4462,10 @@
         <x:v>You</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>Needs Pinterest profile and designs</x:v>
+        <x:v>Use assets/pins/week-01 and publish no more than two per day</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
@@ -4490,7 +4490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R231f82648b8c4dde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aefd696f9394c9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4775,7 +4775,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf96c643d4adb48dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71f624013cea4da8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record first published Pinterest Pin
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R317fda558bce403f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Ra84ee8a9aded4499"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rdad84725b95248c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R4f8664acaae941df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="Rdfcdb76975034703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4c39240990164680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Ra341c6e37fe64bb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="R6526a04b4bd749a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R40f38405a0d442e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R49c1d274b3cd480e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd13a5605df244d07"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R79945bc8b2024663"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -551,7 +551,7 @@
       </x:c>
       <x:c r="B5" t="n">
         <x:f>COUNTIF(Pins!G2:G61,"Published")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Daily cadence</x:v>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31cb536d6e3646d1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4de11b70e65049cd"/>
 </x:worksheet>
 </file>
 
@@ -800,10 +800,14 @@
         <x:v>small apartment organization</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
-        <x:v>Planned</x:v>
-      </x:c>
-      <x:c r="H2" s="9" t="str"/>
-      <x:c r="I2" s="9" t="str"/>
+        <x:v>Published</x:v>
+      </x:c>
+      <x:c r="H2" s="9" t="str">
+        <x:v>https://www.pinterest.com/pin/1132233162595139388/</x:v>
+      </x:c>
+      <x:c r="I2" s="9" t="str">
+        <x:v>https://tidysmallspaces.github.io/guides/no-drill-storage.html</x:v>
+      </x:c>
       <x:c r="J2" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -825,7 +829,9 @@
       <x:c r="P2" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q2" s="9" t="str"/>
+      <x:c r="Q2" s="9" t="str">
+        <x:v>First organic Pin published.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="9" t="str">
@@ -3608,7 +3614,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca9ec2e7bca14c52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb023261b2323446a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4285,7 +4291,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R373d89abc9354cd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R772418d0e31344b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4490,7 +4496,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aefd696f9394c9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69dcad2262de4f23"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4775,7 +4781,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71f624013cea4da8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf090b4d24aa64c46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Separate scheduled Pins from future ideas
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4c39240990164680"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Ra341c6e37fe64bb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="R6526a04b4bd749a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R40f38405a0d442e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R49c1d274b3cd480e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R92e542f4d8524530"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Ra74e2a24bd0c4f81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="R6ccb282b79a34a8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="Rbcd1f30ea22e4307"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="Rb52065bbeb0e48af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R79945bc8b2024663"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9192ef3362024347"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4de11b70e65049cd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ea8f70357734444"/>
 </x:worksheet>
 </file>
 
@@ -3614,7 +3614,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb023261b2323446a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccf92497664f4499"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4291,7 +4291,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R772418d0e31344b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R574b9fc0ce1a4156"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4468,10 +4468,10 @@
         <x:v>You</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>Use assets/pins/week-01 and publish no more than two per day</x:v>
+        <x:v>Scheduled across five days at two Pins per day</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
@@ -4496,7 +4496,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69dcad2262de4f23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d5fbefe3ad342f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4781,7 +4781,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf090b4d24aa64c46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7616a28c54344586"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record Amazon Associates activation
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R92e542f4d8524530"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Ra74e2a24bd0c4f81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="R6ccb282b79a34a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="Rbcd1f30ea22e4307"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="Rb52065bbeb0e48af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4c4155298db54c41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Re3aafe469a864fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="R21bba62ffe3c4cd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="Rc426e50d99bc439e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R3bf03e3bc0024138"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9192ef3362024347"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6008c623e9a3419b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ea8f70357734444"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb063759e124e40fb"/>
 </x:worksheet>
 </file>
 
@@ -3614,7 +3614,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccf92497664f4499"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d616cc456774670"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4291,7 +4291,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R574b9fc0ce1a4156"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb519477872f646b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4412,24 +4412,24 @@
         <x:v>You</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Do after website is public</x:v>
+        <x:v>Associate ID: tidysmallspac-20</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="9" t="str">
-        <x:v>Register website and Pinterest profile in Associates</x:v>
+        <x:v>Register website in Associates</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
         <x:v>You</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>Needs both public URLs</x:v>
+        <x:v>Registered website: tidysmallspaces.github.io</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
@@ -4440,10 +4440,10 @@
         <x:v>Together</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>Only create links inside Associates</x:v>
+        <x:v>Create product links with SiteStripe using tidysmallspac-20</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -4496,7 +4496,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d5fbefe3ad342f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reffc3aa2255b4ef8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4781,7 +4781,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7616a28c54344586"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdc8c68206b24695"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Amazon product-link intake workflow
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4c4155298db54c41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Re3aafe469a864fae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="R21bba62ffe3c4cd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="Rc426e50d99bc439e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R3bf03e3bc0024138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1ca6c0a55f7f41cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Rde4b40c4992d4e97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rc9668e53fd3049b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R267f1e9faa094bc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="Reafd874ad93b46e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6008c623e9a3419b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4a8f61c77d39456f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -324,7 +324,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SetupTable" displayName="SetupTable" ref="A1:D13" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SetupTable" displayName="SetupTable" ref="A1:D14" headerRowCount="1">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Step"/>
     <x:tableColumn id="2" name="Owner"/>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb063759e124e40fb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26ad5f84f6a84272"/>
 </x:worksheet>
 </file>
 
@@ -3614,7 +3614,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d616cc456774670"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79942344faaa44ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4291,7 +4291,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb519477872f646b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4242832cd1c4e01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4434,69 +4434,83 @@
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="9" t="str">
-        <x:v>Add Associates tag links to guides</x:v>
+        <x:v>Complete Amazon payment and tax setup</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>Together</x:v>
+        <x:v>You</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>Create product links with SiteStripe using tidysmallspac-20</x:v>
+        <x:v>Tax interview completed</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="9" t="str">
-        <x:v>Create first weekly Pin batch</x:v>
+        <x:v>Add Associates tag links to guides</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Together</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>Done</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>10 upload-ready PNGs plus editable SVG sources</x:v>
+        <x:v>Create product links with SiteStripe using tidysmallspac-20</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
       <x:c r="A12" s="9" t="str">
-        <x:v>Schedule first 10 Pins in Pinterest</x:v>
+        <x:v>Create first weekly Pin batch</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str">
-        <x:v>You</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>Scheduled across five days at two Pins per day</x:v>
+        <x:v>10 upload-ready PNGs plus editable SVG sources</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
       <x:c r="A13" s="9" t="str">
+        <x:v>Schedule first 10 Pins in Pinterest</x:v>
+      </x:c>
+      <x:c r="B13" s="9" t="str">
+        <x:v>You</x:v>
+      </x:c>
+      <x:c r="C13" s="9" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D13" s="9" t="str">
+        <x:v>Scheduled across five days at two Pins per day</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="9" t="str">
         <x:v>Review analytics after 14 days</x:v>
       </x:c>
-      <x:c r="B13" s="9" t="str">
+      <x:c r="B14" s="9" t="str">
         <x:v>Together</x:v>
       </x:c>
-      <x:c r="C13" s="9" t="str">
+      <x:c r="C14" s="9" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="D13" s="9" t="str">
+      <x:c r="D14" s="9" t="str">
         <x:v>Use dashboard metrics</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="C2:C13">
+    <x:dataValidation type="list" sqref="C2:C14">
       <x:formula1>"Not started,In progress,Blocked,Done"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reffc3aa2255b4ef8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01710a67e1204348"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4781,7 +4795,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdc8c68206b24695"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95efd7aff1404bd6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record first five-day Pinterest results
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1ca6c0a55f7f41cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Rde4b40c4992d4e97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="Rc9668e53fd3049b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R267f1e9faa094bc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="Reafd874ad93b46e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re96002419fce4c4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Re3324a173c884430"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="R861f9625a6834e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R10f590ee42bd4b4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R89b26a9319c04609"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4a8f61c77d39456f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R68ae745030ac4f26"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -551,7 +551,7 @@
       </x:c>
       <x:c r="B5" t="n">
         <x:f>COUNTIF(Pins!G2:G61,"Published")</x:f>
-        <x:v>1</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Daily cadence</x:v>
@@ -581,7 +581,7 @@
       </x:c>
       <x:c r="B7" t="n">
         <x:f>SUM(Pins!N2:N61)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D7" t="str">
         <x:v>Spend before $30 earned</x:v>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26ad5f84f6a84272"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09391d1ee5b94f06"/>
 </x:worksheet>
 </file>
 
@@ -809,7 +809,7 @@
         <x:v>https://tidysmallspaces.github.io/guides/no-drill-storage.html</x:v>
       </x:c>
       <x:c r="J2" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="K2" s="9" t="n">
         <x:v>0</x:v>
@@ -821,7 +821,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N2" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O2" s="9" t="n">
         <x:v>0</x:v>
@@ -830,7 +830,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q2" s="9" t="str">
-        <x:v>First organic Pin published.</x:v>
+        <x:v>Best engagement: 14 Pin clicks, no outbound clicks.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
@@ -853,12 +853,12 @@
         <x:v>small entryway organization</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str"/>
       <x:c r="I3" s="9" t="str"/>
       <x:c r="J3" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="K3" s="9" t="n">
         <x:v>0</x:v>
@@ -878,7 +878,9 @@
       <x:c r="P3" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q3" s="9" t="str"/>
+      <x:c r="Q3" s="9" t="str">
+        <x:v>Pin clicks: 1; no outbound clicks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="9" t="str">
@@ -900,12 +902,12 @@
         <x:v>under bed storage ideas</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str"/>
       <x:c r="I4" s="9" t="str"/>
       <x:c r="J4" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="K4" s="9" t="n">
         <x:v>0</x:v>
@@ -925,7 +927,9 @@
       <x:c r="P4" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q4" s="9" t="str"/>
+      <x:c r="Q4" s="9" t="str">
+        <x:v>Pin clicks: 0; no outbound clicks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="9" t="str">
@@ -947,12 +951,12 @@
         <x:v>renter friendly storage</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str"/>
       <x:c r="I5" s="9" t="str"/>
       <x:c r="J5" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="K5" s="9" t="n">
         <x:v>0</x:v>
@@ -972,7 +976,9 @@
       <x:c r="P5" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q5" s="9" t="str"/>
+      <x:c r="Q5" s="9" t="str">
+        <x:v>Pin clicks: 0; no outbound clicks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="9" t="str">
@@ -994,12 +1000,12 @@
         <x:v>vertical storage ideas</x:v>
       </x:c>
       <x:c r="G6" s="9" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str"/>
       <x:c r="I6" s="9" t="str"/>
       <x:c r="J6" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K6" s="9" t="n">
         <x:v>0</x:v>
@@ -1019,7 +1025,9 @@
       <x:c r="P6" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q6" s="9" t="str"/>
+      <x:c r="Q6" s="9" t="str">
+        <x:v>Pin clicks: 0; no outbound clicks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="9" t="str">
@@ -1041,12 +1049,12 @@
         <x:v>small space organization</x:v>
       </x:c>
       <x:c r="G7" s="9" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="H7" s="9" t="str"/>
       <x:c r="I7" s="9" t="str"/>
       <x:c r="J7" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="K7" s="9" t="n">
         <x:v>0</x:v>
@@ -1066,7 +1074,9 @@
       <x:c r="P7" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q7" s="9" t="str"/>
+      <x:c r="Q7" s="9" t="str">
+        <x:v>Pin clicks: 0; no outbound clicks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="9" t="str">
@@ -1088,12 +1098,12 @@
         <x:v>small apartment organization</x:v>
       </x:c>
       <x:c r="G8" s="9" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str"/>
       <x:c r="I8" s="9" t="str"/>
       <x:c r="J8" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="K8" s="9" t="n">
         <x:v>0</x:v>
@@ -1113,7 +1123,9 @@
       <x:c r="P8" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q8" s="9" t="str"/>
+      <x:c r="Q8" s="9" t="str">
+        <x:v>Pin clicks: 0; no outbound clicks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="9" t="str">
@@ -1135,12 +1147,12 @@
         <x:v>small entryway organization</x:v>
       </x:c>
       <x:c r="G9" s="9" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="H9" s="9" t="str"/>
       <x:c r="I9" s="9" t="str"/>
       <x:c r="J9" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="K9" s="9" t="n">
         <x:v>0</x:v>
@@ -1160,7 +1172,9 @@
       <x:c r="P9" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q9" s="9" t="str"/>
+      <x:c r="Q9" s="9" t="str">
+        <x:v>Pin clicks: 0; no outbound clicks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="9" t="str">
@@ -1182,12 +1196,12 @@
         <x:v>under bed storage ideas</x:v>
       </x:c>
       <x:c r="G10" s="9" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="H10" s="9" t="str"/>
       <x:c r="I10" s="9" t="str"/>
       <x:c r="J10" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="K10" s="9" t="n">
         <x:v>0</x:v>
@@ -1207,7 +1221,9 @@
       <x:c r="P10" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q10" s="9" t="str"/>
+      <x:c r="Q10" s="9" t="str">
+        <x:v>Pin clicks: 0; no outbound clicks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="9" t="str">
@@ -1229,12 +1245,12 @@
         <x:v>renter friendly storage</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="H11" s="9" t="str"/>
       <x:c r="I11" s="9" t="str"/>
       <x:c r="J11" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K11" s="9" t="n">
         <x:v>0</x:v>
@@ -1254,7 +1270,9 @@
       <x:c r="P11" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q11" s="9" t="str"/>
+      <x:c r="Q11" s="9" t="str">
+        <x:v>Pin clicks: 0; no outbound clicks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="9" t="str">
@@ -3614,7 +3632,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79942344faaa44ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R265bfb20e08a4b20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4291,7 +4309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4242832cd1c4e01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82372c8771904a88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4510,7 +4528,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01710a67e1204348"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc773389be6e4768"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4795,7 +4813,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95efd7aff1404bd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6a0e05e0b6c438c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct first-week Pinterest metrics
</commit_message>
<xml_diff>
--- a/outputs/tidy-small-spaces-tracker.xlsx
+++ b/outputs/tidy-small-spaces-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re96002419fce4c4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="Re3324a173c884430"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="R861f9625a6834e95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R10f590ee42bd4b4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R89b26a9319c04609"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R17b56b0bfb6345f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="2" r:id="R9de110c40b744426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" r:id="R3bdbd7d39ab74f9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" r:id="R6967ea91124c40d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Ideas" sheetId="5" r:id="R4db6c869f8024cba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,7 +270,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R68ae745030ac4f26"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R83d7a87d587546d2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -566,7 +566,7 @@
       </x:c>
       <x:c r="B6" t="n">
         <x:f>SUM(Pins!L2:L61)</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>First review</x:v>
@@ -635,7 +635,7 @@
       </x:c>
       <x:c r="B13" t="n">
         <x:f>SUM(Pins!L2:L15)</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C13" t="n">
         <x:f>SUM(Pins!O2:O15)</x:f>
@@ -700,7 +700,7 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09391d1ee5b94f06"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf821f98c0e104119"/>
 </x:worksheet>
 </file>
 
@@ -809,13 +809,13 @@
         <x:v>https://tidysmallspaces.github.io/guides/no-drill-storage.html</x:v>
       </x:c>
       <x:c r="J2" s="9" t="n">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="K2" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L2" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M2" s="9" t="n">
         <x:v>0</x:v>
@@ -830,7 +830,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q2" s="9" t="str">
-        <x:v>Best engagement: 14 Pin clicks, no outbound clicks.</x:v>
+        <x:v>Best result: 14 Pin clicks and 4 outbound clicks.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
@@ -858,7 +858,7 @@
       <x:c r="H3" s="9" t="str"/>
       <x:c r="I3" s="9" t="str"/>
       <x:c r="J3" s="9" t="n">
-        <x:v>38</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="K3" s="9" t="n">
         <x:v>0</x:v>
@@ -907,7 +907,7 @@
       <x:c r="H4" s="9" t="str"/>
       <x:c r="I4" s="9" t="str"/>
       <x:c r="J4" s="9" t="n">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="K4" s="9" t="n">
         <x:v>0</x:v>
@@ -956,7 +956,7 @@
       <x:c r="H5" s="9" t="str"/>
       <x:c r="I5" s="9" t="str"/>
       <x:c r="J5" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="K5" s="9" t="n">
         <x:v>0</x:v>
@@ -1005,7 +1005,7 @@
       <x:c r="H6" s="9" t="str"/>
       <x:c r="I6" s="9" t="str"/>
       <x:c r="J6" s="9" t="n">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="K6" s="9" t="n">
         <x:v>0</x:v>
@@ -1054,7 +1054,7 @@
       <x:c r="H7" s="9" t="str"/>
       <x:c r="I7" s="9" t="str"/>
       <x:c r="J7" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="K7" s="9" t="n">
         <x:v>0</x:v>
@@ -1103,7 +1103,7 @@
       <x:c r="H8" s="9" t="str"/>
       <x:c r="I8" s="9" t="str"/>
       <x:c r="J8" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="K8" s="9" t="n">
         <x:v>0</x:v>
@@ -1152,7 +1152,7 @@
       <x:c r="H9" s="9" t="str"/>
       <x:c r="I9" s="9" t="str"/>
       <x:c r="J9" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="K9" s="9" t="n">
         <x:v>0</x:v>
@@ -1201,7 +1201,7 @@
       <x:c r="H10" s="9" t="str"/>
       <x:c r="I10" s="9" t="str"/>
       <x:c r="J10" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="K10" s="9" t="n">
         <x:v>0</x:v>
@@ -1250,7 +1250,7 @@
       <x:c r="H11" s="9" t="str"/>
       <x:c r="I11" s="9" t="str"/>
       <x:c r="J11" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K11" s="9" t="n">
         <x:v>0</x:v>
@@ -3632,7 +3632,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R265bfb20e08a4b20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55bad27795d449d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4309,7 +4309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82372c8771904a88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re20e3a02d36c49f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4528,7 +4528,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc773389be6e4768"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R039ae1b0dda64485"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4813,7 +4813,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6a0e05e0b6c438c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43c30cabc9ba40bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>